<commit_message>
feat: Spanish headers and values in the Excel import template
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/inventory-import-sample.xlsx
+++ b/public/templates/inventory-import-sample.xlsx
@@ -473,102 +473,102 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>Título</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>listingType</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>price</t>
+          <t>Precio</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>Moneda</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>Ubicación</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>zone</t>
+          <t>Zona</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>propertyType</t>
+          <t>Tipo</t>
         </is>
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
-          <t>bedrooms</t>
+          <t>Dormitorios</t>
         </is>
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>bathrooms</t>
+          <t>Baños</t>
         </is>
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
-          <t>areaM2</t>
+          <t>Superficie m²</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>yearBuilt</t>
+          <t>Año de construcción</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>features</t>
+          <t>Características</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>amenities</t>
+          <t>Amenidades</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>imageUrl</t>
+          <t>Imagen principal</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>Imágenes</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>Descripción</t>
         </is>
       </c>
       <c r="R1" s="2" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>featured</t>
+          <t>Destacada</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>hero</t>
+          <t>Carrusel principal</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>sale</t>
+          <t>venta</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>casa</t>
         </is>
       </c>
       <c r="I2" s="3" t="n">
@@ -650,14 +650,18 @@
       </c>
       <c r="R2" s="3" t="inlineStr">
         <is>
-          <t>published</t>
-        </is>
-      </c>
-      <c r="S2" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="T2" s="3" t="b">
-        <v>1</v>
+          <t>publicada</t>
+        </is>
+      </c>
+      <c r="S2" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T2" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -669,7 +673,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>sale</t>
+          <t>venta</t>
         </is>
       </c>
       <c r="D3" s="3" t="n">
@@ -692,7 +696,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>apartment</t>
+          <t>apartamento</t>
         </is>
       </c>
       <c r="I3" s="3" t="n">
@@ -730,14 +734,18 @@
       </c>
       <c r="R3" s="3" t="inlineStr">
         <is>
-          <t>published</t>
-        </is>
-      </c>
-      <c r="S3" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="T3" s="3" t="b">
-        <v>0</v>
+          <t>publicada</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -749,7 +757,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>sale</t>
+          <t>venta</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
@@ -772,7 +780,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>land</t>
+          <t>terreno</t>
         </is>
       </c>
       <c r="I4" s="3" t="n">
@@ -800,14 +808,18 @@
       </c>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="S4" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="T4" s="3" t="b">
-        <v>0</v>
+          <t>borrador</t>
+        </is>
+      </c>
+      <c r="S4" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T4" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -819,7 +831,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>rent</t>
+          <t>alquiler</t>
         </is>
       </c>
       <c r="D5" s="3" t="n">
@@ -842,7 +854,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>casa</t>
         </is>
       </c>
       <c r="I5" s="3" t="n">
@@ -876,20 +888,24 @@
       </c>
       <c r="R5" s="3" t="inlineStr">
         <is>
-          <t>published</t>
-        </is>
-      </c>
-      <c r="S5" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="T5" s="3" t="b">
-        <v>0</v>
+          <t>publicada</t>
+        </is>
+      </c>
+      <c r="S5" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T5" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="7">
     <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"sale,rent"</formula1>
+      <formula1>"venta,alquiler"</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"USD,EUR,UYU"</formula1>
@@ -898,16 +914,16 @@
       <formula1>"José Ignacio,Manantiales,La Barra,Península,Mansa"</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"house,apartment,penthouse,land"</formula1>
+      <formula1>"casa,apartamento,penthouse,terreno"</formula1>
     </dataValidation>
     <dataValidation sqref="R2:R500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"published,draft"</formula1>
+      <formula1>"publicada,borrador"</formula1>
     </dataValidation>
     <dataValidation sqref="S2:S500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
+      <formula1>"Sí,No"</formula1>
     </dataValidation>
     <dataValidation sqref="T2:T500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
+      <formula1>"Sí,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -954,7 +970,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
@@ -976,7 +992,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>Título</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -998,7 +1014,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>listingType</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -1013,14 +1029,14 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>sale (venta) | rent (alquiler)</t>
+          <t>venta | alquiler</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>price</t>
+          <t>Precio</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -1042,7 +1058,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>Moneda</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -1064,7 +1080,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>Ubicación</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -1086,7 +1102,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>zone</t>
+          <t>Zona</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -1108,7 +1124,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>propertyType</t>
+          <t>Tipo</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -1123,14 +1139,14 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>house | apartment | penthouse | land</t>
+          <t>casa | apartamento | penthouse | terreno</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>bedrooms</t>
+          <t>Dormitorios</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -1152,7 +1168,7 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>bathrooms</t>
+          <t>Baños</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -1174,7 +1190,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>areaM2</t>
+          <t>Superficie m²</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -1196,7 +1212,7 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>yearBuilt</t>
+          <t>Año de construcción</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -1218,7 +1234,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>features</t>
+          <t>Características</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -1240,7 +1256,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>amenities</t>
+          <t>Amenidades</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -1262,7 +1278,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>imageUrl</t>
+          <t>Imagen principal</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -1284,7 +1300,7 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>Imágenes</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -1306,7 +1322,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>Descripción</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -1328,7 +1344,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -1343,14 +1359,14 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>published | draft</t>
+          <t>publicada | borrador</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>featured</t>
+          <t>Destacada</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -1365,14 +1381,14 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>TRUE | FALSE</t>
+          <t>Sí | No</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>hero</t>
+          <t>Carrusel principal</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -1387,7 +1403,7 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>TRUE | FALSE</t>
+          <t>Sí | No</t>
         </is>
       </c>
     </row>
@@ -1425,14 +1441,14 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>• Listas (features, amenities, images): separá los elementos con punto y coma (;).</t>
+          <t>• Listas (Características, Amenidades, Imágenes): separá los elementos con punto y coma (;).</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>• featured y hero: como máximo 5 propiedades en total para cada una.</t>
+          <t>• Destacada y Carrusel principal: como máximo 5 propiedades en total para cada una.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Cost breakdown, vehicle/real-estate trade-in, and intent priority for leads
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/inventory-import-sample.xlsx
+++ b/public/templates/inventory-import-sample.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T5"/>
+  <dimension ref="A1:V5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -468,6 +468,8 @@
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="11" customWidth="1" min="19" max="19"/>
     <col width="9" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -571,6 +573,16 @@
           <t>Carrusel principal</t>
         </is>
       </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Gastos comunes</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Impuestos</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -662,6 +674,12 @@
         <is>
           <t>Sí</t>
         </is>
+      </c>
+      <c r="U2" s="3" t="n">
+        <v>650</v>
+      </c>
+      <c r="V2" s="3" t="n">
+        <v>4800</v>
       </c>
     </row>
     <row r="3">
@@ -746,6 +764,12 @@
         <is>
           <t>No</t>
         </is>
+      </c>
+      <c r="U3" s="3" t="n">
+        <v>280</v>
+      </c>
+      <c r="V3" s="3" t="n">
+        <v>1500</v>
       </c>
     </row>
     <row r="4">
@@ -821,6 +845,8 @@
           <t>No</t>
         </is>
       </c>
+      <c r="U4" s="3" t="inlineStr"/>
+      <c r="V4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr"/>
@@ -900,6 +926,12 @@
         <is>
           <t>No</t>
         </is>
+      </c>
+      <c r="U5" s="3" t="n">
+        <v>280</v>
+      </c>
+      <c r="V5" s="3" t="n">
+        <v>1500</v>
       </c>
     </row>
   </sheetData>
@@ -936,7 +968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1408,52 +1440,96 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Gastos comunes</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Gastos comunes mensuales, en la moneda de la propiedad. Se muestran en el desglose de costos.</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Número ≥ 0</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Impuestos</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Impuestos anuales (contribución inmobiliaria, primaria), en la moneda de la propiedad.</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Número ≥ 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>Notas</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>• Los encabezados de la hoja «Inventario» (fila 1) no deben cambiarse; el orden de las columnas no importa.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>• Las columnas con encabezado rojo son obligatorias.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>• Las filas de ejemplo se pueden borrar o reemplazar.</t>
+          <t>• Los encabezados de la hoja «Inventario» (fila 1) no deben cambiarse; el orden de las columnas no importa.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>• Listas (Características, Amenidades, Imágenes): separá los elementos con punto y coma (;).</t>
+          <t>• Las columnas con encabezado rojo son obligatorias.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>• Destacada y Carrusel principal: como máximo 5 propiedades en total para cada una.</t>
+          <t>• Las filas de ejemplo se pueden borrar o reemplazar.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
+        <is>
+          <t>• Listas (Características, Amenidades, Imágenes): separá los elementos con punto y coma (;).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>• Destacada y Carrusel principal: como máximo 5 propiedades en total para cada una.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
         <is>
           <t>• Guardá el archivo como .xlsx.</t>
         </is>

</xml_diff>